<commit_message>
feat: comprehensive update - web dashboard, interactive tag review, and parsing fixesImplemented Flask web dashboard with drag-and-drop uploadAdded interactive non-numeric tag review system (Phase 1 Scan)Enhanced measurement parsing to handle common typos (double dots, commas)Added red highlighting for unparseable rows in output for manual correctionImproved fabric normalization and deduction extractionAdded template generation and verification utility scripts
</commit_message>
<xml_diff>
--- a/rb2.xlsx
+++ b/rb2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mdash\Downloads\Excel clean\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mdash\Downloads\Excel-clean\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E95D3A82-629C-4E4A-BBCA-BD57F877621B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F7CC30E-5A23-4AC7-B56C-0AB022682403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8C2F2230-33F4-424C-BED6-B0E404033255}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="38">
   <si>
     <t>Project:</t>
   </si>
@@ -151,6 +151,9 @@
   </si>
   <si>
     <t>Deducts D=1/2</t>
+  </si>
+  <si>
+    <t>DR</t>
   </si>
 </sst>
 </file>
@@ -1166,7 +1169,7 @@
         <v>14</v>
       </c>
       <c r="F10" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">

</xml_diff>